<commit_message>
bug fix, menos falsos positivos
</commit_message>
<xml_diff>
--- a/Reporte_Eventos_Seguridad.xlsx
+++ b/Reporte_Eventos_Seguridad.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,6 +808,1414 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EVT-AED62891E64A4EA597365EE94990F37C</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>14:23:15.441</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.917</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_142315_436_4990F37C.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EVT-4D2FDA81163647A59CE04BA28BBABACF</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>14:23:15.754</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Falta Chaleco</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_142315_754_8BBABACF.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EVT-ED05E274ADFD40BAA2C4F2366BC159C3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>14:24:14.449</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_142414_433_6BC159C3.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EVT-9562B71FC5CB4EE1AB539CADC96F5FA2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>14:24:17.283</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Falta Chaleco</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_142417_268_C96F5FA2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EVT-7CB73F3492AA45FBBEE7333F4D8D510E</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>14:30:07.793</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143007_793_4D8D510E.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EVT-AD26EBC539EA4F17B879EB15573E1369</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>14:30:56.015</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143056_015_573E1369.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>EVT-7F53A32EF2894CE3BB1DF62984E59881</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>14:31:09.157</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143109_157_84E59881.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EVT-D830EF2C1DB844E0A2C1DBF1B9CB7CA2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>14:31:42.789</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143142_789_B9CB7CA2.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>EVT-E53AFFDD52BE4C5DAB8BEBF02D03CD4C</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>14:32:15.841</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Falta Chaleco</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0.917</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143215_837_2D03CD4C.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EVT-BE060CA38EF14AB5A13706226672332D</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>14:32:19.680</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143219_680_6672332D.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EVT-12F09BCD14494E4B9127F64A1EB7040D</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>14:32:23.426</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143223_426_1EB7040D.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EVT-3AAB0E555CCF452886CDD842D84C7A48</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>14:32:47.596</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143247_592_D84C7A48.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>EVT-9419A0F240A1424EAD6C17EDE31449C9</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>14:32:48.742</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143248_734_E31449C9.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EVT-A62C655C94624253AD9058034C2A3E1B</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>14:32:52.323</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>POSIBLE_CAIDA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_POSIBLE_CAIDA_20260724_143252_323_4C2A3E1B.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>EVT-7FF806AA430B4D35ADE852D50814AC86</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>14:32:52.745</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143252_740_0814AC86.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EVT-16B2E071222243CA95E66D1550820F92</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>14:33:20.705</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>0.917</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143320_689_50820F92.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>EVT-43A4EA9D4A784AB7AD79B8A993813F8D</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>14:34:21.865</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143421_865_93813F8D.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EVT-2ACFCD1C20F94C1C8525B848A4EA57F9</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>14:34:23.314</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143423_299_A4EA57F9.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>EVT-598EB4CF8ACE469A8393CE4D5D57DF14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>14:35:07.673</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143507_673_5D57DF14.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>EVT-A22B641A9AA74B2C91F20569003072FC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>14:35:09.324</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143509_324_003072FC.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>EVT-1BA332B2149B4CFDAABDC0BFD6CA5F71</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>14:35:09.340</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>POSIBLE_CAIDA</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Falta Casco</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_POSIBLE_CAIDA_20260724_143509_324_D6CA5F71.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EVT-95AEDF5C8EAE4519B8AD2AD97E919E7F</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>CAM_PUERTA01_ADM_CONCENTRADORA</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>14:38:36.868</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>INCUMPLIMIENTO_EPP</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Sin Casco y Chaleco</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Evidencias\CAM_PUERTA01_ADM_CONCENTRADORA_INCUMPLIMIENTO_EPP_20260724_143836_866_7E919E7F.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mejoras en la documentación y ajustes en la carga de variables de entorno; se agrega prueba para verificar la carga del archivo .env.
</commit_message>
<xml_diff>
--- a/Reporte_Eventos_Seguridad.xlsx
+++ b/Reporte_Eventos_Seguridad.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,72 +429,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Evento_ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Camara</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Tipo_Evento</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Casco</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Chaleco</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Estado_EPP</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Confianza_Evento</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ID_Seguimiento_Temporal</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Estado_Revision</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Identificacion_Humana</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Observaciones_Revision</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Foto</t>
         </is>

</xml_diff>